<commit_message>
here for the standard_user we have done the login , with the valid credentials,with blank password,and the incorrect password and for all of the case the result is pass
</commit_message>
<xml_diff>
--- a/src/TestData/UITesting.xlsx
+++ b/src/TestData/UITesting.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{783DEFBA-45F4-4E36-84D0-A7F49494DDBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11430" windowHeight="3570" firstSheet="1" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="shreya" sheetId="1" r:id="rId1"/>
@@ -13,7 +12,8 @@
     <sheet name="shreyash" sheetId="3" r:id="rId3"/>
     <sheet name="ayush" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A14:D22"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1113,7 +1113,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5">
     <font>
       <sz val="11"/>
@@ -1496,7 +1496,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1787,7 +1787,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A776755-8DBA-4DB1-BBEC-F133E32FB1EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
@@ -2423,7 +2423,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA40B599-1E19-4741-941B-AA096A48A848}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3215,19 +3215,19 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C24" r:id="rId1" xr:uid="{8BC969EE-33AD-42E2-A462-5726F472E87D}"/>
-    <hyperlink ref="C25" r:id="rId2" xr:uid="{1B5E84FB-D4E1-4460-AA1E-CB0E88E24EC8}"/>
-    <hyperlink ref="C26" r:id="rId3" xr:uid="{40121F2D-9FB5-46D4-9A35-DC2A1C5ED79B}"/>
-    <hyperlink ref="C27" r:id="rId4" xr:uid="{E81EDEA4-1C19-4E90-A799-DEBC04E58134}"/>
-    <hyperlink ref="C28" r:id="rId5" display="Sauce Labs Bolt T-Shirt" xr:uid="{0BC66F8C-4F5C-4680-8145-608558DCFEE8}"/>
-    <hyperlink ref="C29" r:id="rId6" xr:uid="{E36827CC-4333-4F7E-AD60-957BBD8F4CA5}"/>
+    <hyperlink ref="C24" r:id="rId1"/>
+    <hyperlink ref="C25" r:id="rId2"/>
+    <hyperlink ref="C26" r:id="rId3"/>
+    <hyperlink ref="C27" r:id="rId4"/>
+    <hyperlink ref="C28" r:id="rId5" display="Sauce Labs Bolt T-Shirt"/>
+    <hyperlink ref="C29" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B13F163D-67AE-4E5C-AFEA-95C00C151A04}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3738,7 +3738,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.75">
+    <row r="20" spans="1:8">
       <c r="A20" s="3" t="s">
         <v>318</v>
       </c>
@@ -3961,11 +3961,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D11" r:id="rId1" xr:uid="{2000FC39-D95B-477F-A5B2-A6B6CB112966}"/>
-    <hyperlink ref="D12" r:id="rId2" xr:uid="{2905889D-6420-49B3-9F09-066B64B012BE}"/>
-    <hyperlink ref="D13" r:id="rId3" xr:uid="{9A439393-3C8C-4C82-870B-3464E7D7758D}"/>
-    <hyperlink ref="D14" r:id="rId4" xr:uid="{8C668141-09ED-4A38-BBC8-2459CF91CC45}"/>
-    <hyperlink ref="D15" r:id="rId5" xr:uid="{9EC8835E-EC5D-4E43-8A62-27D986C55768}"/>
+    <hyperlink ref="D11" r:id="rId1"/>
+    <hyperlink ref="D12" r:id="rId2"/>
+    <hyperlink ref="D13" r:id="rId3"/>
+    <hyperlink ref="D14" r:id="rId4"/>
+    <hyperlink ref="D15" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
aqll the test files
</commit_message>
<xml_diff>
--- a/src/TestData/UITesting.xlsx
+++ b/src/TestData/UITesting.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{783DEFBA-45F4-4E36-84D0-A7F49494DDBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/38fbe1cab3a1115b/Desktop/CRC_devops/Project/Devops-saucedemo/src/TestData/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:801_{2C450DB4-F661-4D20-9045-60E4D1A7BEBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69199752-D406-469D-8B8E-D75C58A90EED}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="shreya" sheetId="1" r:id="rId1"/>
@@ -13,21 +18,10 @@
     <sheet name="shreyash" sheetId="3" r:id="rId3"/>
     <sheet name="ayush" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -1114,7 +1108,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1169,7 +1163,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1181,7 +1175,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1201,9 +1194,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1241,7 +1234,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1347,7 +1340,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1489,7 +1482,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1498,19 +1491,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.109375" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="4" max="4" width="51.140625" customWidth="1"/>
+    <col min="4" max="4" width="51.109375" customWidth="1"/>
     <col min="5" max="5" width="68" customWidth="1"/>
-    <col min="6" max="6" width="61.7109375" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" customWidth="1"/>
-    <col min="9" max="9" width="60.7109375" customWidth="1"/>
+    <col min="6" max="6" width="61.6640625" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" customWidth="1"/>
+    <col min="9" max="9" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1539,7 +1532,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1568,7 +1561,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1597,7 +1590,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -1626,7 +1619,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -1655,8 +1648,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>37</v>
       </c>
       <c r="B6" t="s">
@@ -1684,7 +1677,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1694,7 +1687,7 @@
       <c r="C7" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" t="s">
         <v>47</v>
       </c>
       <c r="E7" t="s">
@@ -1713,7 +1706,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>51</v>
       </c>
@@ -1742,7 +1735,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>58</v>
       </c>
@@ -1771,12 +1764,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>65</v>
       </c>
@@ -1789,17 +1782,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A776755-8DBA-4DB1-BBEC-F133E32FB1EC}">
   <dimension ref="A1:I27"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="47.5703125" customWidth="1"/>
-    <col min="4" max="4" width="36.42578125" customWidth="1"/>
-    <col min="5" max="5" width="31.5703125" customWidth="1"/>
-    <col min="6" max="6" width="42.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" customWidth="1"/>
+    <col min="3" max="3" width="47.5546875" customWidth="1"/>
+    <col min="4" max="4" width="36.44140625" customWidth="1"/>
+    <col min="5" max="5" width="31.5546875" customWidth="1"/>
+    <col min="6" max="6" width="42.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1828,7 +1821,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1851,7 +1844,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1874,7 +1867,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1897,7 +1890,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1920,7 +1913,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1943,7 +1936,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1966,7 +1959,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1989,7 +1982,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2012,7 +2005,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2035,7 +2028,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2058,7 +2051,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2081,7 +2074,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2104,7 +2097,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2127,7 +2120,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2150,7 +2143,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2173,7 +2166,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2196,7 +2189,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2219,7 +2212,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2242,7 +2235,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2265,7 +2258,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2288,7 +2281,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2311,7 +2304,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2334,7 +2327,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2357,7 +2350,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2380,7 +2373,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2403,7 +2396,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2425,18 +2418,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA40B599-1E19-4741-941B-AA096A48A848}">
   <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="36.28515625" customWidth="1"/>
-    <col min="4" max="4" width="51.42578125" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="36.33203125" customWidth="1"/>
+    <col min="4" max="4" width="51.44140625" customWidth="1"/>
+    <col min="5" max="5" width="27.44140625" customWidth="1"/>
     <col min="6" max="6" width="32" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>158</v>
       </c>
@@ -2465,7 +2458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>159</v>
       </c>
@@ -2494,7 +2487,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="17.25" customHeight="1">
+    <row r="3" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -2520,7 +2513,7 @@
         <v>46243</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -2546,7 +2539,7 @@
         <v>46243</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -2569,7 +2562,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -2592,7 +2585,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -2615,7 +2608,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>51</v>
       </c>
@@ -2638,7 +2631,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="17.25" customHeight="1">
+    <row r="9" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>58</v>
       </c>
@@ -2664,7 +2657,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -2687,7 +2680,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>65</v>
       </c>
@@ -2710,7 +2703,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>185</v>
       </c>
@@ -2733,7 +2726,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>189</v>
       </c>
@@ -2756,7 +2749,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>193</v>
       </c>
@@ -2779,7 +2772,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>197</v>
       </c>
@@ -2802,7 +2795,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>201</v>
       </c>
@@ -2825,7 +2818,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>206</v>
       </c>
@@ -2848,7 +2841,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>210</v>
       </c>
@@ -2871,7 +2864,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>213</v>
       </c>
@@ -2894,7 +2887,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>218</v>
       </c>
@@ -2917,7 +2910,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>222</v>
       </c>
@@ -2940,7 +2933,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>225</v>
       </c>
@@ -2963,7 +2956,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>228</v>
       </c>
@@ -2986,7 +2979,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>232</v>
       </c>
@@ -3009,7 +3002,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>235</v>
       </c>
@@ -3032,7 +3025,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>238</v>
       </c>
@@ -3055,7 +3048,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>241</v>
       </c>
@@ -3078,7 +3071,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>243</v>
       </c>
@@ -3101,7 +3094,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>245</v>
       </c>
@@ -3124,7 +3117,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>247</v>
       </c>
@@ -3147,7 +3140,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>250</v>
       </c>
@@ -3170,7 +3163,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>252</v>
       </c>
@@ -3193,22 +3186,22 @@
         <v>161</v>
       </c>
     </row>
-    <row r="33" spans="1:1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="35" spans="1:1">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="36" spans="1:1">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>257</v>
       </c>
@@ -3229,19 +3222,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B13F163D-67AE-4E5C-AFEA-95C00C151A04}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
     <col min="3" max="3" width="36" customWidth="1"/>
-    <col min="4" max="4" width="29.42578125" customWidth="1"/>
-    <col min="5" max="5" width="41.7109375" customWidth="1"/>
+    <col min="4" max="4" width="29.44140625" customWidth="1"/>
+    <col min="5" max="5" width="41.6640625" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="16384" max="16384" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="16384" max="16384" width="9.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>158</v>
       </c>
@@ -3270,7 +3263,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>258</v>
       </c>
@@ -3296,7 +3289,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>264</v>
       </c>
@@ -3322,7 +3315,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>267</v>
       </c>
@@ -3348,7 +3341,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>270</v>
       </c>
@@ -3374,7 +3367,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>274</v>
       </c>
@@ -3400,7 +3393,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>279</v>
       </c>
@@ -3426,7 +3419,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>283</v>
       </c>
@@ -3452,7 +3445,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>286</v>
       </c>
@@ -3478,7 +3471,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>289</v>
       </c>
@@ -3504,7 +3497,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>293</v>
       </c>
@@ -3530,7 +3523,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>297</v>
       </c>
@@ -3556,7 +3549,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>298</v>
       </c>
@@ -3582,7 +3575,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>299</v>
       </c>
@@ -3608,7 +3601,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="14.25" customHeight="1">
+    <row r="15" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>300</v>
       </c>
@@ -3634,7 +3627,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1">
+    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>301</v>
       </c>
@@ -3660,7 +3653,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>306</v>
       </c>
@@ -3686,7 +3679,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>311</v>
       </c>
@@ -3712,7 +3705,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>315</v>
       </c>
@@ -3738,7 +3731,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.75">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>318</v>
       </c>
@@ -3764,7 +3757,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>320</v>
       </c>
@@ -3790,7 +3783,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>324</v>
       </c>
@@ -3816,7 +3809,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>329</v>
       </c>
@@ -3842,7 +3835,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>333</v>
       </c>
@@ -3868,7 +3861,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>337</v>
       </c>
@@ -3894,7 +3887,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>342</v>
       </c>
@@ -3920,7 +3913,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>346</v>
       </c>
@@ -3946,7 +3939,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>350</v>
       </c>
@@ -3954,7 +3947,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>352</v>
       </c>

</xml_diff>